<commit_message>
bets.py sheet logs by default; week 4 data and reconstructed bet log
- sheet now logs a batch unless --no-log is passed (--log still accepted);
  README, WEEKLY.md updated
- nfl_bets/data/bet_log.csv: week 4 batch reconstructed after the fact from
  the 09-30 Kalshi and 10-02 sportsbook snapshots (sheet was run without
  --log), graded; rows carry a note column saying so
- week 4 Kalshi closing snapshots, pool picks log, action splits, weekly lines

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/nfl_model/data/weekly_lines.xlsx
+++ b/nfl_model/data/weekly_lines.xlsx
@@ -2697,13 +2697,13 @@
         </is>
       </c>
       <c r="L50" t="n">
-        <v>-1.5</v>
+        <v>-0.5</v>
       </c>
       <c r="M50" t="n">
-        <v>39.5</v>
+        <v>40</v>
       </c>
       <c r="N50" t="n">
-        <v>0.528</v>
+        <v>0.506</v>
       </c>
     </row>
     <row r="51">
@@ -2754,10 +2754,10 @@
         <v>2.5</v>
       </c>
       <c r="M51" t="n">
-        <v>46</v>
+        <v>46.5</v>
       </c>
       <c r="N51" t="n">
-        <v>0.43</v>
+        <v>0.438</v>
       </c>
     </row>
     <row r="52">
@@ -2797,10 +2797,10 @@
         </is>
       </c>
       <c r="L52" t="n">
-        <v>-11</v>
+        <v>-10.5</v>
       </c>
       <c r="M52" t="n">
-        <v>46</v>
+        <v>46.5</v>
       </c>
       <c r="N52" t="n">
         <v>0.8129999999999999</v>
@@ -2843,13 +2843,13 @@
         </is>
       </c>
       <c r="L53" t="n">
-        <v>-5</v>
+        <v>-4.5</v>
       </c>
       <c r="M53" t="n">
-        <v>47</v>
+        <v>46.5</v>
       </c>
       <c r="N53" t="n">
-        <v>0.657</v>
+        <v>0.642</v>
       </c>
     </row>
     <row r="54">
@@ -2889,13 +2889,13 @@
         </is>
       </c>
       <c r="L54" t="n">
-        <v>-3.5</v>
+        <v>-3</v>
       </c>
       <c r="M54" t="n">
         <v>41.5</v>
       </c>
       <c r="N54" t="n">
-        <v>0.629</v>
+        <v>0.596</v>
       </c>
     </row>
     <row r="55">
@@ -2935,13 +2935,13 @@
         </is>
       </c>
       <c r="L55" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="M55" t="n">
-        <v>49.5</v>
+        <v>50.5</v>
       </c>
       <c r="N55" t="n">
-        <v>0.522</v>
+        <v>0.486</v>
       </c>
     </row>
     <row r="56">
@@ -2992,10 +2992,10 @@
         <v>-4</v>
       </c>
       <c r="M56" t="n">
-        <v>48.5</v>
+        <v>49</v>
       </c>
       <c r="N56" t="n">
-        <v>0.641</v>
+        <v>0.642</v>
       </c>
     </row>
     <row r="57">
@@ -3046,10 +3046,10 @@
         <v>-2</v>
       </c>
       <c r="M57" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N57" t="n">
-        <v>0.547</v>
+        <v>0.537</v>
       </c>
     </row>
     <row r="58">
@@ -3097,13 +3097,13 @@
         </is>
       </c>
       <c r="L58" t="n">
-        <v>-3.5</v>
+        <v>-2.5</v>
       </c>
       <c r="M58" t="n">
-        <v>45.5</v>
+        <v>46</v>
       </c>
       <c r="N58" t="n">
-        <v>0.613</v>
+        <v>0.5649999999999999</v>
       </c>
     </row>
     <row r="59">
@@ -3124,7 +3124,7 @@
         <v>3.5</v>
       </c>
       <c r="E59" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="F59" t="n">
         <v>1.5</v>
@@ -3151,13 +3151,13 @@
         </is>
       </c>
       <c r="L59" t="n">
-        <v>-1</v>
+        <v>3</v>
       </c>
       <c r="M59" t="n">
-        <v>47</v>
+        <v>43.5</v>
       </c>
       <c r="N59" t="n">
-        <v>0.509</v>
+        <v>0.407</v>
       </c>
     </row>
     <row r="60">
@@ -3178,7 +3178,7 @@
         <v>-11.5</v>
       </c>
       <c r="E60" t="n">
-        <v>-10.5</v>
+        <v>-10</v>
       </c>
       <c r="F60" t="n">
         <v>-10.5</v>
@@ -3205,13 +3205,13 @@
         </is>
       </c>
       <c r="L60" t="n">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="M60" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="N60" t="n">
-        <v>0.745</v>
+        <v>0.779</v>
       </c>
     </row>
     <row r="61">
@@ -3251,13 +3251,13 @@
         </is>
       </c>
       <c r="L61" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="M61" t="n">
         <v>47.5</v>
       </c>
       <c r="N61" t="n">
-        <v>0.328</v>
+        <v>0.339</v>
       </c>
     </row>
     <row r="62">
@@ -3297,13 +3297,13 @@
         </is>
       </c>
       <c r="L62" t="n">
-        <v>-7.5</v>
+        <v>-8</v>
       </c>
       <c r="M62" t="n">
         <v>41</v>
       </c>
       <c r="N62" t="n">
-        <v>0.756</v>
+        <v>0.778</v>
       </c>
     </row>
     <row r="63">
@@ -3354,10 +3354,10 @@
         <v>-3</v>
       </c>
       <c r="M63" t="n">
-        <v>47.5</v>
+        <v>48</v>
       </c>
       <c r="N63" t="n">
-        <v>0.573</v>
+        <v>0.601</v>
       </c>
     </row>
     <row r="64">
@@ -3405,13 +3405,13 @@
         </is>
       </c>
       <c r="L64" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="M64" t="n">
-        <v>48.5</v>
+        <v>49</v>
       </c>
       <c r="N64" t="n">
-        <v>0.376</v>
+        <v>0.369</v>
       </c>
     </row>
     <row r="65">
@@ -3432,7 +3432,7 @@
         <v>-2.5</v>
       </c>
       <c r="E65" t="n">
-        <v>-2.5</v>
+        <v>-1.5</v>
       </c>
       <c r="F65" t="n">
         <v>-2.5</v>
@@ -3454,10 +3454,10 @@
         <v>-2.5</v>
       </c>
       <c r="M65" t="n">
-        <v>46.5</v>
+        <v>46</v>
       </c>
       <c r="N65" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Week 5 data: pool picks and splits, Claude's picks, ELWAY bet log, Kalshi snapshots
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/nfl_model/data/weekly_lines.xlsx
+++ b/nfl_model/data/weekly_lines.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N65"/>
+  <dimension ref="A1:N80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3460,6 +3460,696 @@
         <v>0.57</v>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>5</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>TB</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>-9.5</v>
+      </c>
+      <c r="E66" t="n">
+        <v>-9.5</v>
+      </c>
+      <c r="F66" t="n">
+        <v>-9.5</v>
+      </c>
+      <c r="G66" t="n">
+        <v>73</v>
+      </c>
+      <c r="H66" t="n">
+        <v>70</v>
+      </c>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-09T18:34</t>
+        </is>
+      </c>
+      <c r="L66" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="M66" t="n">
+        <v>50</v>
+      </c>
+      <c r="N66" t="n">
+        <v>0.707</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>5</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>JAX</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="E67" t="n">
+        <v>-7.5</v>
+      </c>
+      <c r="F67" t="n">
+        <v>-2</v>
+      </c>
+      <c r="G67" t="n">
+        <v>61</v>
+      </c>
+      <c r="H67" t="n">
+        <v>57</v>
+      </c>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-09T18:34</t>
+        </is>
+      </c>
+      <c r="L67" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="M67" t="n">
+        <v>46</v>
+      </c>
+      <c r="N67" t="n">
+        <v>0.634</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>5</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E68" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F68" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="G68" t="n">
+        <v>43</v>
+      </c>
+      <c r="H68" t="n">
+        <v>55</v>
+      </c>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-09T18:34</t>
+        </is>
+      </c>
+      <c r="L68" t="n">
+        <v>-3</v>
+      </c>
+      <c r="M68" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="N68" t="n">
+        <v>0.604</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>5</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>CIN</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="E69" t="n">
+        <v>7</v>
+      </c>
+      <c r="F69" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="G69" t="n">
+        <v>25</v>
+      </c>
+      <c r="H69" t="n">
+        <v>14</v>
+      </c>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-09T18:34</t>
+        </is>
+      </c>
+      <c r="L69" t="n">
+        <v>5</v>
+      </c>
+      <c r="M69" t="n">
+        <v>46</v>
+      </c>
+      <c r="N69" t="n">
+        <v>0.335</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>5</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>LV</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="E70" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="F70" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="G70" t="n">
+        <v>29</v>
+      </c>
+      <c r="H70" t="n">
+        <v>24</v>
+      </c>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-09T18:34</t>
+        </is>
+      </c>
+      <c r="L70" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="M70" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="N70" t="n">
+        <v>0.723</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>5</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E71" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F71" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G71" t="n">
+        <v>45</v>
+      </c>
+      <c r="H71" t="n">
+        <v>48</v>
+      </c>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-09T18:34</t>
+        </is>
+      </c>
+      <c r="L71" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="M71" t="n">
+        <v>43</v>
+      </c>
+      <c r="N71" t="n">
+        <v>0.462</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>5</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>CLE</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>NYJ</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="E72" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="F72" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="G72" t="n">
+        <v>16</v>
+      </c>
+      <c r="H72" t="n">
+        <v>26</v>
+      </c>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-09T18:34</t>
+        </is>
+      </c>
+      <c r="L72" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="M72" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="N72" t="n">
+        <v>0.435</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>5</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>IND</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="E73" t="n">
+        <v>-3</v>
+      </c>
+      <c r="F73" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="G73" t="n">
+        <v>35</v>
+      </c>
+      <c r="H73" t="n">
+        <v>39</v>
+      </c>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-09T18:34</t>
+        </is>
+      </c>
+      <c r="L73" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="M73" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="N73" t="n">
+        <v>0.548</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>5</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>HOU</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>TEN</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E74" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="F74" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G74" t="n">
+        <v>29</v>
+      </c>
+      <c r="H74" t="n">
+        <v>35</v>
+      </c>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-09T18:34</t>
+        </is>
+      </c>
+      <c r="L74" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="M74" t="n">
+        <v>41</v>
+      </c>
+      <c r="N74" t="n">
+        <v>0.283</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>5</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>NYG</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>WAS</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="E75" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="F75" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="G75" t="n">
+        <v>26</v>
+      </c>
+      <c r="H75" t="n">
+        <v>25</v>
+      </c>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-09T18:34</t>
+        </is>
+      </c>
+      <c r="L75" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="M75" t="n">
+        <v>44</v>
+      </c>
+      <c r="N75" t="n">
+        <v>0.531</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>5</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>DEN</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>LAC</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E76" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F76" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G76" t="n">
+        <v>45</v>
+      </c>
+      <c r="H76" t="n">
+        <v>46</v>
+      </c>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-09T18:34</t>
+        </is>
+      </c>
+      <c r="L76" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="M76" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="N76" t="n">
+        <v>0.441</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>5</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>ARI</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E77" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="F77" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="G77" t="n">
+        <v>45</v>
+      </c>
+      <c r="H77" t="n">
+        <v>44</v>
+      </c>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-09T18:34</t>
+        </is>
+      </c>
+      <c r="L77" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M77" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="N77" t="n">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>5</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="E78" t="n">
+        <v>-3</v>
+      </c>
+      <c r="F78" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="G78" t="n">
+        <v>19</v>
+      </c>
+      <c r="H78" t="n">
+        <v>13</v>
+      </c>
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-09T18:34</t>
+        </is>
+      </c>
+      <c r="L78" t="n">
+        <v>-3</v>
+      </c>
+      <c r="M78" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="N78" t="n">
+        <v>0.576</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>5</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>BAL</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="E79" t="n">
+        <v>-3</v>
+      </c>
+      <c r="F79" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G79" t="n">
+        <v>47</v>
+      </c>
+      <c r="H79" t="n">
+        <v>56</v>
+      </c>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-09T18:34</t>
+        </is>
+      </c>
+      <c r="L79" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="M79" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="N79" t="n">
+        <v>0.571</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>5</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>BUF</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>LAR</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="E80" t="n">
+        <v>-3</v>
+      </c>
+      <c r="F80" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="G80" t="n">
+        <v>27</v>
+      </c>
+      <c r="H80" t="n">
+        <v>40</v>
+      </c>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-09T18:34</t>
+        </is>
+      </c>
+      <c r="L80" t="n">
+        <v>-3</v>
+      </c>
+      <c r="M80" t="n">
+        <v>53</v>
+      </c>
+      <c r="N80" t="n">
+        <v>0.575</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weeks 6-7 data: pool lines and ELWAY imports, splits, picks, ELWAY bet log, Kalshi snapshots
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/nfl_model/data/weekly_lines.xlsx
+++ b/nfl_model/data/weekly_lines.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N80"/>
+  <dimension ref="A1:N108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4150,6 +4150,1154 @@
         <v>0.575</v>
       </c>
     </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>6</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>DEN</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E81" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F81" t="n">
+        <v>2</v>
+      </c>
+      <c r="G81" t="n">
+        <v>41</v>
+      </c>
+      <c r="H81" t="n">
+        <v>38</v>
+      </c>
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-18T13:59</t>
+        </is>
+      </c>
+      <c r="L81" t="n">
+        <v>1</v>
+      </c>
+      <c r="M81" t="n">
+        <v>41</v>
+      </c>
+      <c r="N81" t="n">
+        <v>0.476</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>6</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>HOU</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>JAX</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="E82" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="F82" t="n">
+        <v>-3</v>
+      </c>
+      <c r="G82" t="n">
+        <v>50</v>
+      </c>
+      <c r="H82" t="n">
+        <v>48</v>
+      </c>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-18T13:59</t>
+        </is>
+      </c>
+      <c r="L82" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="M82" t="n">
+        <v>43</v>
+      </c>
+      <c r="N82" t="n">
+        <v>0.5580000000000001</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>6</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E83" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F83" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G83" t="n">
+        <v>58</v>
+      </c>
+      <c r="H83" t="n">
+        <v>60</v>
+      </c>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-18T13:59</t>
+        </is>
+      </c>
+      <c r="L83" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="M83" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="N83" t="n">
+        <v>0.533</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>6</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>BAL</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>CLE</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E84" t="n">
+        <v>3</v>
+      </c>
+      <c r="F84" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G84" t="n">
+        <v>44</v>
+      </c>
+      <c r="H84" t="n">
+        <v>46</v>
+      </c>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-18T13:59</t>
+        </is>
+      </c>
+      <c r="L84" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="M84" t="n">
+        <v>43</v>
+      </c>
+      <c r="N84" t="n">
+        <v>0.374</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>6</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>TEN</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>IND</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>-7.5</v>
+      </c>
+      <c r="E85" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="F85" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="G85" t="n">
+        <v>77</v>
+      </c>
+      <c r="H85" t="n">
+        <v>83</v>
+      </c>
+      <c r="I85" t="inlineStr"/>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-18T13:59</t>
+        </is>
+      </c>
+      <c r="L85" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="M85" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="N85" t="n">
+        <v>0.717</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>6</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>NYJ</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>-7.5</v>
+      </c>
+      <c r="E86" t="n">
+        <v>-7.5</v>
+      </c>
+      <c r="F86" t="n">
+        <v>-7</v>
+      </c>
+      <c r="G86" t="n">
+        <v>76</v>
+      </c>
+      <c r="H86" t="n">
+        <v>71</v>
+      </c>
+      <c r="I86" t="inlineStr"/>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-18T13:59</t>
+        </is>
+      </c>
+      <c r="L86" t="n">
+        <v>-8.5</v>
+      </c>
+      <c r="M86" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="N86" t="n">
+        <v>0.787</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>6</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>NYG</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E87" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F87" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G87" t="n">
+        <v>55</v>
+      </c>
+      <c r="H87" t="n">
+        <v>59</v>
+      </c>
+      <c r="I87" t="inlineStr"/>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-18T13:59</t>
+        </is>
+      </c>
+      <c r="L87" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="M87" t="n">
+        <v>44</v>
+      </c>
+      <c r="N87" t="n">
+        <v>0.5649999999999999</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>6</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="E88" t="n">
+        <v>3</v>
+      </c>
+      <c r="F88" t="n">
+        <v>-2</v>
+      </c>
+      <c r="G88" t="n">
+        <v>40</v>
+      </c>
+      <c r="H88" t="n">
+        <v>30</v>
+      </c>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>mkt_line = 9-book median PK on Oct 14 (books CAR -1.5 to PHI -1.5; nflverse had CAR -1.5); Action Network splits 2026-10-18T13:59</t>
+        </is>
+      </c>
+      <c r="L88" t="n">
+        <v>-3</v>
+      </c>
+      <c r="M88" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="N88" t="n">
+        <v>0.604</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>6</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>TB</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E89" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F89" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G89" t="n">
+        <v>33</v>
+      </c>
+      <c r="H89" t="n">
+        <v>37</v>
+      </c>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-18T13:59</t>
+        </is>
+      </c>
+      <c r="L89" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="M89" t="n">
+        <v>41</v>
+      </c>
+      <c r="N89" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>6</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>ARI</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>LAR</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>-12.5</v>
+      </c>
+      <c r="E90" t="n">
+        <v>-12.5</v>
+      </c>
+      <c r="F90" t="n">
+        <v>-10.5</v>
+      </c>
+      <c r="G90" t="n">
+        <v>74</v>
+      </c>
+      <c r="H90" t="n">
+        <v>75</v>
+      </c>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-18T13:59</t>
+        </is>
+      </c>
+      <c r="L90" t="n">
+        <v>-7.5</v>
+      </c>
+      <c r="M90" t="n">
+        <v>51</v>
+      </c>
+      <c r="N90" t="n">
+        <v>0.749</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>6</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>LAC</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>KC</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>-8.5</v>
+      </c>
+      <c r="E91" t="n">
+        <v>-7.5</v>
+      </c>
+      <c r="F91" t="n">
+        <v>-7.5</v>
+      </c>
+      <c r="G91" t="n">
+        <v>68</v>
+      </c>
+      <c r="H91" t="n">
+        <v>64</v>
+      </c>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-18T13:59</t>
+        </is>
+      </c>
+      <c r="L91" t="n">
+        <v>-10.5</v>
+      </c>
+      <c r="M91" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="N91" t="n">
+        <v>0.8110000000000001</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>6</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>BUF</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>LV</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="E92" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="F92" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G92" t="n">
+        <v>33</v>
+      </c>
+      <c r="H92" t="n">
+        <v>37</v>
+      </c>
+      <c r="I92" t="inlineStr"/>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-18T13:59</t>
+        </is>
+      </c>
+      <c r="L92" t="n">
+        <v>5</v>
+      </c>
+      <c r="M92" t="n">
+        <v>50</v>
+      </c>
+      <c r="N92" t="n">
+        <v>0.339</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>6</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="E93" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="F93" t="n">
+        <v>1</v>
+      </c>
+      <c r="G93" t="n">
+        <v>38</v>
+      </c>
+      <c r="H93" t="n">
+        <v>36</v>
+      </c>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-18T13:59</t>
+        </is>
+      </c>
+      <c r="L93" t="n">
+        <v>-3</v>
+      </c>
+      <c r="M93" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="N93" t="n">
+        <v>0.588</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>6</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>WAS</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>-7.5</v>
+      </c>
+      <c r="E94" t="n">
+        <v>-7.5</v>
+      </c>
+      <c r="F94" t="n">
+        <v>-7.5</v>
+      </c>
+      <c r="G94" t="n">
+        <v>79</v>
+      </c>
+      <c r="H94" t="n">
+        <v>85</v>
+      </c>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-18T13:59</t>
+        </is>
+      </c>
+      <c r="L94" t="n">
+        <v>-11</v>
+      </c>
+      <c r="M94" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="N94" t="n">
+        <v>0.8149999999999999</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>7</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="E95" t="n">
+        <v>-3</v>
+      </c>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr"/>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="n">
+        <v>-1</v>
+      </c>
+      <c r="M95" t="n">
+        <v>48</v>
+      </c>
+      <c r="N95" t="n">
+        <v>0.514</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>7</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E96" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="n">
+        <v>3</v>
+      </c>
+      <c r="M96" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="N96" t="n">
+        <v>0.403</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>7</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>ATL</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E97" t="n">
+        <v>3</v>
+      </c>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="n">
+        <v>3</v>
+      </c>
+      <c r="M97" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="N97" t="n">
+        <v>0.395</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>7</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>CIN</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>BAL</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E98" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr"/>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr"/>
+      <c r="L98" t="n">
+        <v>-3</v>
+      </c>
+      <c r="M98" t="n">
+        <v>51</v>
+      </c>
+      <c r="N98" t="n">
+        <v>0.595</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>7</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>TB</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="E99" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr"/>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="M99" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="N99" t="n">
+        <v>0.531</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>7</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>NYG</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>HOU</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>-10.5</v>
+      </c>
+      <c r="E100" t="n">
+        <v>-10.5</v>
+      </c>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr"/>
+      <c r="H100" t="inlineStr"/>
+      <c r="I100" t="inlineStr"/>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" t="n">
+        <v>-7</v>
+      </c>
+      <c r="M100" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="N100" t="n">
+        <v>0.749</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>7</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>IND</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="E101" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr"/>
+      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr"/>
+      <c r="J101" t="inlineStr"/>
+      <c r="K101" t="inlineStr"/>
+      <c r="L101" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="M101" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="N101" t="n">
+        <v>0.712</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>7</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>MIA</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>NYJ</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="E102" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr"/>
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr"/>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr"/>
+      <c r="L102" t="n">
+        <v>-2</v>
+      </c>
+      <c r="M102" t="n">
+        <v>41</v>
+      </c>
+      <c r="N102" t="n">
+        <v>0.547</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>7</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>CLE</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>TEN</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E103" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F103" t="inlineStr"/>
+      <c r="G103" t="inlineStr"/>
+      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr"/>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr"/>
+      <c r="L103" t="n">
+        <v>2</v>
+      </c>
+      <c r="M103" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="N103" t="n">
+        <v>0.456</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>7</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>DEN</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>ARI</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E104" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F104" t="inlineStr"/>
+      <c r="G104" t="inlineStr"/>
+      <c r="H104" t="inlineStr"/>
+      <c r="I104" t="inlineStr"/>
+      <c r="J104" t="inlineStr"/>
+      <c r="K104" t="inlineStr"/>
+      <c r="L104" t="n">
+        <v>4</v>
+      </c>
+      <c r="M104" t="n">
+        <v>46</v>
+      </c>
+      <c r="N104" t="n">
+        <v>0.362</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>7</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="E105" t="n">
+        <v>-3</v>
+      </c>
+      <c r="F105" t="inlineStr"/>
+      <c r="G105" t="inlineStr"/>
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr"/>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr"/>
+      <c r="L105" t="n">
+        <v>-5</v>
+      </c>
+      <c r="M105" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="N105" t="n">
+        <v>0.656</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>7</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>LAR</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>LV</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E106" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr"/>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr"/>
+      <c r="L106" t="n">
+        <v>3</v>
+      </c>
+      <c r="M106" t="n">
+        <v>50</v>
+      </c>
+      <c r="N106" t="n">
+        <v>0.407</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>7</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>KC</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="E107" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr"/>
+      <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr"/>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr"/>
+      <c r="L107" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="M107" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="N107" t="n">
+        <v>0.622</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>7</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E108" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="inlineStr"/>
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr"/>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr"/>
+      <c r="L108" t="n">
+        <v>1</v>
+      </c>
+      <c r="M108" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="N108" t="n">
+        <v>0.478</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Week 7 data: betting splits and the workbook's splits columns
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/nfl_model/data/weekly_lines.xlsx
+++ b/nfl_model/data/weekly_lines.xlsx
@@ -4814,12 +4814,22 @@
       <c r="E95" t="n">
         <v>-3</v>
       </c>
-      <c r="F95" t="inlineStr"/>
-      <c r="G95" t="inlineStr"/>
-      <c r="H95" t="inlineStr"/>
+      <c r="F95" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="G95" t="n">
+        <v>33</v>
+      </c>
+      <c r="H95" t="n">
+        <v>37</v>
+      </c>
       <c r="I95" t="inlineStr"/>
       <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-23T14:08</t>
+        </is>
+      </c>
       <c r="L95" t="n">
         <v>-1</v>
       </c>
@@ -4848,14 +4858,24 @@
         <v>3.5</v>
       </c>
       <c r="E96" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="F96" t="inlineStr"/>
-      <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="F96" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G96" t="n">
+        <v>56</v>
+      </c>
+      <c r="H96" t="n">
+        <v>59</v>
+      </c>
       <c r="I96" t="inlineStr"/>
       <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-23T14:08</t>
+        </is>
+      </c>
       <c r="L96" t="n">
         <v>3</v>
       </c>
@@ -4884,14 +4904,24 @@
         <v>3.5</v>
       </c>
       <c r="E97" t="n">
-        <v>3</v>
-      </c>
-      <c r="F97" t="inlineStr"/>
-      <c r="G97" t="inlineStr"/>
-      <c r="H97" t="inlineStr"/>
+        <v>2.5</v>
+      </c>
+      <c r="F97" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G97" t="n">
+        <v>28</v>
+      </c>
+      <c r="H97" t="n">
+        <v>42</v>
+      </c>
       <c r="I97" t="inlineStr"/>
       <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-23T14:08</t>
+        </is>
+      </c>
       <c r="L97" t="n">
         <v>3</v>
       </c>
@@ -4920,14 +4950,24 @@
         <v>1.5</v>
       </c>
       <c r="E98" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="F98" t="inlineStr"/>
-      <c r="G98" t="inlineStr"/>
-      <c r="H98" t="inlineStr"/>
+        <v>-1.5</v>
+      </c>
+      <c r="F98" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="G98" t="n">
+        <v>28</v>
+      </c>
+      <c r="H98" t="n">
+        <v>20</v>
+      </c>
       <c r="I98" t="inlineStr"/>
       <c r="J98" t="inlineStr"/>
-      <c r="K98" t="inlineStr"/>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-23T14:08</t>
+        </is>
+      </c>
       <c r="L98" t="n">
         <v>-3</v>
       </c>
@@ -4956,14 +4996,24 @@
         <v>-3.5</v>
       </c>
       <c r="E99" t="n">
-        <v>-3.5</v>
-      </c>
-      <c r="F99" t="inlineStr"/>
-      <c r="G99" t="inlineStr"/>
-      <c r="H99" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="F99" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="G99" t="n">
+        <v>64</v>
+      </c>
+      <c r="H99" t="n">
+        <v>39</v>
+      </c>
       <c r="I99" t="inlineStr"/>
       <c r="J99" t="inlineStr"/>
-      <c r="K99" t="inlineStr"/>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-23T14:08</t>
+        </is>
+      </c>
       <c r="L99" t="n">
         <v>-1.5</v>
       </c>
@@ -4994,12 +5044,22 @@
       <c r="E100" t="n">
         <v>-10.5</v>
       </c>
-      <c r="F100" t="inlineStr"/>
-      <c r="G100" t="inlineStr"/>
-      <c r="H100" t="inlineStr"/>
+      <c r="F100" t="n">
+        <v>-7.5</v>
+      </c>
+      <c r="G100" t="n">
+        <v>36</v>
+      </c>
+      <c r="H100" t="n">
+        <v>51</v>
+      </c>
       <c r="I100" t="inlineStr"/>
       <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr"/>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-23T14:08</t>
+        </is>
+      </c>
       <c r="L100" t="n">
         <v>-7</v>
       </c>
@@ -5030,12 +5090,22 @@
       <c r="E101" t="n">
         <v>-6.5</v>
       </c>
-      <c r="F101" t="inlineStr"/>
-      <c r="G101" t="inlineStr"/>
-      <c r="H101" t="inlineStr"/>
+      <c r="F101" t="n">
+        <v>-5.5</v>
+      </c>
+      <c r="G101" t="n">
+        <v>47</v>
+      </c>
+      <c r="H101" t="n">
+        <v>39</v>
+      </c>
       <c r="I101" t="inlineStr"/>
       <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-23T14:08</t>
+        </is>
+      </c>
       <c r="L101" t="n">
         <v>-6.5</v>
       </c>
@@ -5066,12 +5136,22 @@
       <c r="E102" t="n">
         <v>-4.5</v>
       </c>
-      <c r="F102" t="inlineStr"/>
-      <c r="G102" t="inlineStr"/>
-      <c r="H102" t="inlineStr"/>
+      <c r="F102" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="G102" t="n">
+        <v>52</v>
+      </c>
+      <c r="H102" t="n">
+        <v>42</v>
+      </c>
       <c r="I102" t="inlineStr"/>
       <c r="J102" t="inlineStr"/>
-      <c r="K102" t="inlineStr"/>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-23T14:08</t>
+        </is>
+      </c>
       <c r="L102" t="n">
         <v>-2</v>
       </c>
@@ -5102,12 +5182,22 @@
       <c r="E103" t="n">
         <v>1.5</v>
       </c>
-      <c r="F103" t="inlineStr"/>
-      <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr"/>
+      <c r="F103" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G103" t="n">
+        <v>29</v>
+      </c>
+      <c r="H103" t="n">
+        <v>46</v>
+      </c>
       <c r="I103" t="inlineStr"/>
       <c r="J103" t="inlineStr"/>
-      <c r="K103" t="inlineStr"/>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-23T14:08</t>
+        </is>
+      </c>
       <c r="L103" t="n">
         <v>2</v>
       </c>
@@ -5138,12 +5228,22 @@
       <c r="E104" t="n">
         <v>4.5</v>
       </c>
-      <c r="F104" t="inlineStr"/>
-      <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr"/>
+      <c r="F104" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="G104" t="n">
+        <v>39</v>
+      </c>
+      <c r="H104" t="n">
+        <v>32</v>
+      </c>
       <c r="I104" t="inlineStr"/>
       <c r="J104" t="inlineStr"/>
-      <c r="K104" t="inlineStr"/>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-23T14:08</t>
+        </is>
+      </c>
       <c r="L104" t="n">
         <v>4</v>
       </c>
@@ -5174,12 +5274,22 @@
       <c r="E105" t="n">
         <v>-3</v>
       </c>
-      <c r="F105" t="inlineStr"/>
-      <c r="G105" t="inlineStr"/>
-      <c r="H105" t="inlineStr"/>
+      <c r="F105" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="G105" t="n">
+        <v>33</v>
+      </c>
+      <c r="H105" t="n">
+        <v>28</v>
+      </c>
       <c r="I105" t="inlineStr"/>
       <c r="J105" t="inlineStr"/>
-      <c r="K105" t="inlineStr"/>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-23T14:08</t>
+        </is>
+      </c>
       <c r="L105" t="n">
         <v>-5</v>
       </c>
@@ -5208,14 +5318,24 @@
         <v>4.5</v>
       </c>
       <c r="E106" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="F106" t="inlineStr"/>
-      <c r="G106" t="inlineStr"/>
-      <c r="H106" t="inlineStr"/>
+        <v>3.5</v>
+      </c>
+      <c r="F106" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G106" t="n">
+        <v>61</v>
+      </c>
+      <c r="H106" t="n">
+        <v>64</v>
+      </c>
       <c r="I106" t="inlineStr"/>
       <c r="J106" t="inlineStr"/>
-      <c r="K106" t="inlineStr"/>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-23T14:08</t>
+        </is>
+      </c>
       <c r="L106" t="n">
         <v>3</v>
       </c>
@@ -5244,14 +5364,24 @@
         <v>-2.5</v>
       </c>
       <c r="E107" t="n">
-        <v>-2.5</v>
-      </c>
-      <c r="F107" t="inlineStr"/>
-      <c r="G107" t="inlineStr"/>
-      <c r="H107" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="F107" t="n">
+        <v>-2</v>
+      </c>
+      <c r="G107" t="n">
+        <v>11</v>
+      </c>
+      <c r="H107" t="n">
+        <v>11</v>
+      </c>
       <c r="I107" t="inlineStr"/>
       <c r="J107" t="inlineStr"/>
-      <c r="K107" t="inlineStr"/>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-23T14:08</t>
+        </is>
+      </c>
       <c r="L107" t="n">
         <v>-3.5</v>
       </c>
@@ -5282,12 +5412,22 @@
       <c r="E108" t="n">
         <v>4.5</v>
       </c>
-      <c r="F108" t="inlineStr"/>
-      <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
+      <c r="F108" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G108" t="n">
+        <v>33</v>
+      </c>
+      <c r="H108" t="n">
+        <v>30</v>
+      </c>
       <c r="I108" t="inlineStr"/>
       <c r="J108" t="inlineStr"/>
-      <c r="K108" t="inlineStr"/>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Action Network splits 2026-10-23T14:08</t>
+        </is>
+      </c>
       <c r="L108" t="n">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Week 7 data: graded ELWAY bets (and week 6's MNF), Kalshi snapshots, pool picks and splits, Claude's picks
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/nfl_model/data/weekly_lines.xlsx
+++ b/nfl_model/data/weekly_lines.xlsx
@@ -4880,10 +4880,10 @@
         <v>3</v>
       </c>
       <c r="M96" t="n">
-        <v>43.5</v>
+        <v>43</v>
       </c>
       <c r="N96" t="n">
-        <v>0.403</v>
+        <v>0.421</v>
       </c>
     </row>
     <row r="97">
@@ -4923,13 +4923,13 @@
         </is>
       </c>
       <c r="L97" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="M97" t="n">
         <v>49.5</v>
       </c>
       <c r="N97" t="n">
-        <v>0.395</v>
+        <v>0.389</v>
       </c>
     </row>
     <row r="98">
@@ -4950,7 +4950,7 @@
         <v>1.5</v>
       </c>
       <c r="E98" t="n">
-        <v>-1.5</v>
+        <v>3</v>
       </c>
       <c r="F98" t="n">
         <v>-3.5</v>
@@ -4972,10 +4972,10 @@
         <v>-3</v>
       </c>
       <c r="M98" t="n">
-        <v>51</v>
+        <v>51.5</v>
       </c>
       <c r="N98" t="n">
-        <v>0.595</v>
+        <v>0.596</v>
       </c>
     </row>
     <row r="99">
@@ -5015,13 +5015,13 @@
         </is>
       </c>
       <c r="L99" t="n">
-        <v>-1.5</v>
+        <v>-0.5</v>
       </c>
       <c r="M99" t="n">
-        <v>46.5</v>
+        <v>47</v>
       </c>
       <c r="N99" t="n">
-        <v>0.531</v>
+        <v>0.508</v>
       </c>
     </row>
     <row r="100">
@@ -5042,7 +5042,7 @@
         <v>-10.5</v>
       </c>
       <c r="E100" t="n">
-        <v>-10.5</v>
+        <v>-10</v>
       </c>
       <c r="F100" t="n">
         <v>-7.5</v>
@@ -5067,7 +5067,7 @@
         <v>45.5</v>
       </c>
       <c r="N100" t="n">
-        <v>0.749</v>
+        <v>0.739</v>
       </c>
     </row>
     <row r="101">
@@ -5110,10 +5110,10 @@
         <v>-6.5</v>
       </c>
       <c r="M101" t="n">
-        <v>44.5</v>
+        <v>45</v>
       </c>
       <c r="N101" t="n">
-        <v>0.712</v>
+        <v>0.716</v>
       </c>
     </row>
     <row r="102">
@@ -5134,7 +5134,7 @@
         <v>-4.5</v>
       </c>
       <c r="E102" t="n">
-        <v>-4.5</v>
+        <v>-3.5</v>
       </c>
       <c r="F102" t="n">
         <v>-4.5</v>
@@ -5156,10 +5156,10 @@
         <v>-2</v>
       </c>
       <c r="M102" t="n">
-        <v>41</v>
+        <v>42.5</v>
       </c>
       <c r="N102" t="n">
-        <v>0.547</v>
+        <v>0.542</v>
       </c>
     </row>
     <row r="103">
@@ -5199,13 +5199,13 @@
         </is>
       </c>
       <c r="L103" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="M103" t="n">
-        <v>40.5</v>
+        <v>40</v>
       </c>
       <c r="N103" t="n">
-        <v>0.456</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="104">
@@ -5245,13 +5245,13 @@
         </is>
       </c>
       <c r="L104" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="M104" t="n">
-        <v>46</v>
+        <v>45.5</v>
       </c>
       <c r="N104" t="n">
-        <v>0.362</v>
+        <v>0.347</v>
       </c>
     </row>
     <row r="105">
@@ -5272,7 +5272,7 @@
         <v>-2.5</v>
       </c>
       <c r="E105" t="n">
-        <v>-3</v>
+        <v>-3.5</v>
       </c>
       <c r="F105" t="n">
         <v>-3.5</v>
@@ -5291,13 +5291,13 @@
         </is>
       </c>
       <c r="L105" t="n">
-        <v>-5</v>
+        <v>-5.5</v>
       </c>
       <c r="M105" t="n">
-        <v>53.5</v>
+        <v>54</v>
       </c>
       <c r="N105" t="n">
-        <v>0.656</v>
+        <v>0.666</v>
       </c>
     </row>
     <row r="106">
@@ -5343,7 +5343,7 @@
         <v>50</v>
       </c>
       <c r="N106" t="n">
-        <v>0.407</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="107">
@@ -5389,7 +5389,7 @@
         <v>43.5</v>
       </c>
       <c r="N107" t="n">
-        <v>0.622</v>
+        <v>0.633</v>
       </c>
     </row>
     <row r="108">
@@ -5432,10 +5432,10 @@
         <v>1</v>
       </c>
       <c r="M108" t="n">
-        <v>48.5</v>
+        <v>49</v>
       </c>
       <c r="N108" t="n">
-        <v>0.478</v>
+        <v>0.473</v>
       </c>
     </row>
   </sheetData>

</xml_diff>